<commit_message>
Se agrega persistencia con Mysql
Se agrega persistencia con Mysql
</commit_message>
<xml_diff>
--- a/RiskEventNotifacionBackend/ProjectStructure.xlsx
+++ b/RiskEventNotifacionBackend/ProjectStructure.xlsx
@@ -12,7 +12,8 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12450"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Proyect_Backend" sheetId="1" r:id="rId1"/>
+    <sheet name="BaseDatos_Model" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="78">
   <si>
     <t>RiskEventNotifacion.Api</t>
   </si>
@@ -219,13 +220,52 @@
   </si>
   <si>
     <t>DataSource</t>
+  </si>
+  <si>
+    <t>Tablas</t>
+  </si>
+  <si>
+    <t>usuarioChannels</t>
+  </si>
+  <si>
+    <t>usuarios</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>userrname</t>
+  </si>
+  <si>
+    <t>estado</t>
+  </si>
+  <si>
+    <t>IdUsuario</t>
+  </si>
+  <si>
+    <t>sms</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>push</t>
+  </si>
+  <si>
+    <t>whatsapp</t>
+  </si>
+  <si>
+    <t>IDataSource</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -251,6 +291,12 @@
       <color rgb="FF00B050"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF2B91AF"/>
+      <name val="Cascadia Mono"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="3">
@@ -294,12 +340,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -311,6 +354,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -605,305 +654,307 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="3" t="s">
+      <c r="B1" s="8"/>
+      <c r="C1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="7" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="6" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="5"/>
-      <c r="B8" s="7" t="s">
+      <c r="A8" s="4"/>
+      <c r="B8" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="5"/>
-      <c r="B9" s="4" t="s">
+      <c r="A9" s="4"/>
+      <c r="B9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="6" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="5"/>
-      <c r="B10" s="7" t="s">
+      <c r="A10" s="4"/>
+      <c r="B10" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="4"/>
+      <c r="B11" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="5"/>
-      <c r="B11" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="E11" s="7" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="4"/>
+      <c r="B12" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="5"/>
-      <c r="B12" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E12" s="4" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="4"/>
+      <c r="B13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="5"/>
-      <c r="B13" s="4" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="4"/>
+      <c r="B14" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="4"/>
+      <c r="B15" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="5"/>
-      <c r="B14" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="E14" s="4" t="s">
+      <c r="E15" s="3" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="5"/>
-      <c r="B15" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" s="5"/>
-    </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="5"/>
-      <c r="B16" s="7" t="s">
+      <c r="A16" s="4"/>
+      <c r="B16" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="E16" s="5"/>
+      <c r="E16" s="4"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="7" t="s">
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="E17" s="5"/>
+      <c r="E17" s="4"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -912,4 +963,70 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="11.42578125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>